<commit_message>
updated xls and E67 files
</commit_message>
<xml_diff>
--- a/aysha/FittingTests.xlsx
+++ b/aysha/FittingTests.xlsx
@@ -1,31 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\tamuq-chen-secarelab-receiver\aysha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6AF479-A372-48EC-A6DA-56BB467FC295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D4B5AC-AB60-4A36-B381-850C8AC2677E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="0D" sheetId="1" r:id="rId1"/>
+    <sheet name="3D" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="87">
   <si>
     <t>A</t>
   </si>
@@ -118,6 +131,174 @@
   </si>
   <si>
     <t>no convergence</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>as close as possible to E67</t>
+  </si>
+  <si>
+    <t>v7</t>
+  </si>
+  <si>
+    <t>conjugated</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>temperature appeared too low</t>
+  </si>
+  <si>
+    <t>Raytracing</t>
+  </si>
+  <si>
+    <t>changed power x8 to achieve Power on apperture equal to all other cases</t>
+  </si>
+  <si>
+    <t>profile improved significantly but too high</t>
+  </si>
+  <si>
+    <t>power x4 incase the 1/4 symmetry creates the issues</t>
+  </si>
+  <si>
+    <t>agreement got better not ideal</t>
+  </si>
+  <si>
+    <t>no correction as original E67 without the 0.64</t>
+  </si>
+  <si>
+    <t>Heat</t>
+  </si>
+  <si>
+    <t>Cps x 4</t>
+  </si>
+  <si>
+    <t>too low</t>
+  </si>
+  <si>
+    <t>too high</t>
+  </si>
+  <si>
+    <t>added 4x on Psrc</t>
+  </si>
+  <si>
+    <t>back to Cps</t>
+  </si>
+  <si>
+    <t>repeated x4 on Psrc and 0.64 on Io</t>
+  </si>
+  <si>
+    <t>again to high</t>
+  </si>
+  <si>
+    <t>changed to x2</t>
+  </si>
+  <si>
+    <t>removed 0.64, and changed h_nat=10</t>
+  </si>
+  <si>
+    <t>corrected V0 to qlpm/4 to account for 1/4 symmetry</t>
+  </si>
+  <si>
+    <t>added 0.64, h_nat=1, and 1.87x Psrc to match total absorbed power</t>
+  </si>
+  <si>
+    <t>promising results, T3 very good time series, T-length not bad, pasted pictures to Aysha</t>
+  </si>
+  <si>
+    <t>overal temperature reduced, and profile didn’t get better</t>
+  </si>
+  <si>
+    <t>initial of 3b, 1 min</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>broadening C limit didn't help</t>
+  </si>
+  <si>
+    <t>C limit to 30</t>
+  </si>
+  <si>
+    <t>corrected m(qlpm, Tamb) and G flux in Re</t>
+  </si>
+  <si>
+    <t>2. x Psrc</t>
+  </si>
+  <si>
+    <t>not bad, but solid not great, modeled is higher, also very strange behavior for Nu because of Pr</t>
+  </si>
+  <si>
+    <t>changed Pr expressin to fixed Tamb</t>
+  </si>
+  <si>
+    <t>gas slightly lower, solid slight higher</t>
+  </si>
+  <si>
+    <t>gas all lower, gas better but all slightly higher</t>
+  </si>
+  <si>
+    <t>similar</t>
+  </si>
+  <si>
+    <t>Cp</t>
+  </si>
+  <si>
+    <t>scatter plot ok but solid profiles not</t>
+  </si>
+  <si>
+    <t>scatter plot worse and solid profiles not</t>
+  </si>
+  <si>
+    <t>gas scatter and profiles ok, solid not</t>
+  </si>
+  <si>
+    <t>solid profiles better than gas</t>
+  </si>
+  <si>
+    <t>init #26, changed limits of A B C</t>
+  </si>
+  <si>
+    <t>RH</t>
+  </si>
+  <si>
+    <t>change limits for C</t>
+  </si>
+  <si>
+    <t>reworked some of the inputs to be able for non-isothermal flow; poor</t>
+  </si>
+  <si>
+    <t>T9-T10</t>
+  </si>
+  <si>
+    <t>had trouble to repeat #9, deactivated multi-physics for surface radiation</t>
+  </si>
+  <si>
+    <t>same as #9, w 2xPsrc</t>
+  </si>
+  <si>
+    <t>too high temperature</t>
+  </si>
+  <si>
+    <t>1.6Psrc</t>
+  </si>
+  <si>
+    <t>gave a good agreement on the Length Profilel</t>
+  </si>
+  <si>
+    <t>1.4x</t>
+  </si>
+  <si>
+    <t>hnat=10</t>
+  </si>
+  <si>
+    <t>better match but not at all points</t>
+  </si>
+  <si>
+    <t>try to change the front temperature</t>
   </si>
 </sst>
 </file>
@@ -125,7 +306,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -165,13 +346,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,13 +636,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:M14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:O37"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="13" max="13" width="46.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="46.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -490,13 +674,19 @@
         <v>27</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -531,13 +721,19 @@
         <v>28</v>
       </c>
       <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>0.4</v>
+      </c>
+      <c r="N3">
         <v>499.47699999999998</v>
       </c>
-      <c r="M3" t="s">
+      <c r="O3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -553,14 +749,14 @@
       <c r="E4">
         <v>0.66</v>
       </c>
-      <c r="L4">
+      <c r="N4">
         <v>528.26599999999996</v>
       </c>
-      <c r="M4" t="s">
+      <c r="O4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -579,14 +775,14 @@
       <c r="F5">
         <v>1</v>
       </c>
-      <c r="L5">
+      <c r="N5">
         <v>473.34</v>
       </c>
-      <c r="M5" t="s">
+      <c r="O5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -602,11 +798,11 @@
       <c r="G6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="M6" t="s">
+      <c r="O6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -622,14 +818,14 @@
       <c r="G7">
         <v>1</v>
       </c>
-      <c r="L7">
+      <c r="N7">
         <v>604.08600000000001</v>
       </c>
-      <c r="M7" t="s">
+      <c r="O7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -645,11 +841,11 @@
       <c r="E8">
         <v>0.7</v>
       </c>
-      <c r="M8" t="s">
+      <c r="O8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -665,11 +861,11 @@
       <c r="E9">
         <v>0.63</v>
       </c>
-      <c r="M9" t="s">
+      <c r="O9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -685,14 +881,14 @@
       <c r="G10">
         <v>1.2</v>
       </c>
-      <c r="L10">
+      <c r="N10">
         <v>500</v>
       </c>
-      <c r="M10" t="s">
+      <c r="O10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -708,14 +904,17 @@
       <c r="E11">
         <v>0.64</v>
       </c>
-      <c r="L11">
+      <c r="N11">
         <v>480</v>
       </c>
-      <c r="M11" t="s">
+      <c r="O11" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>9</v>
+      </c>
       <c r="B12" s="2">
         <v>2.6620817681730501E-5</v>
       </c>
@@ -728,30 +927,669 @@
       <c r="I12" t="s">
         <v>21</v>
       </c>
-      <c r="L12">
+      <c r="N12">
         <v>672</v>
       </c>
-      <c r="M12" t="s">
+      <c r="O12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>10</v>
+      </c>
       <c r="J13" t="s">
         <v>25</v>
       </c>
-      <c r="M13" t="s">
+      <c r="O13" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>11</v>
+      </c>
       <c r="K14" t="s">
         <v>29</v>
       </c>
-      <c r="L14">
+      <c r="N14">
         <v>25612</v>
       </c>
-      <c r="M14" t="s">
+      <c r="O14" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2">
+        <v>3.3035945380220997E-5</v>
+      </c>
+      <c r="C15">
+        <v>1.43770025274668</v>
+      </c>
+      <c r="D15">
+        <v>20</v>
+      </c>
+      <c r="J15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" t="s">
+        <v>28</v>
+      </c>
+      <c r="N15">
+        <v>469</v>
+      </c>
+      <c r="O15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>13</v>
+      </c>
+      <c r="N16" t="s">
+        <v>58</v>
+      </c>
+      <c r="O16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2">
+        <v>1.03191509408719E-5</v>
+      </c>
+      <c r="C17">
+        <v>1.4319313285872399</v>
+      </c>
+      <c r="D17">
+        <v>25.984272299692599</v>
+      </c>
+      <c r="N17">
+        <v>465</v>
+      </c>
+      <c r="O17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>15</v>
+      </c>
+      <c r="O18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>16</v>
+      </c>
+      <c r="E19">
+        <v>0.84</v>
+      </c>
+      <c r="N19">
+        <v>850</v>
+      </c>
+      <c r="O19" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>17</v>
+      </c>
+      <c r="O20" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>18</v>
+      </c>
+      <c r="E21">
+        <v>0.74</v>
+      </c>
+      <c r="F21">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="N21">
+        <v>573</v>
+      </c>
+      <c r="O21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>19</v>
+      </c>
+      <c r="E22">
+        <v>0.64</v>
+      </c>
+      <c r="N22">
+        <v>607</v>
+      </c>
+      <c r="O22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>20</v>
+      </c>
+      <c r="B23">
+        <v>5.6058995390906102E-4</v>
+      </c>
+      <c r="C23">
+        <v>1.6106589591624401</v>
+      </c>
+      <c r="D23">
+        <v>9.910468968988089E-4</v>
+      </c>
+      <c r="E23">
+        <v>0.7</v>
+      </c>
+      <c r="N23">
+        <v>502</v>
+      </c>
+      <c r="O23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>21</v>
+      </c>
+      <c r="B24" s="2">
+        <v>1.0024299213338499E-5</v>
+      </c>
+      <c r="C24">
+        <v>2.9323882617891202</v>
+      </c>
+      <c r="D24">
+        <v>1E-4</v>
+      </c>
+      <c r="L24">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="N24">
+        <v>1641</v>
+      </c>
+      <c r="O24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>22</v>
+      </c>
+      <c r="B25" s="2">
+        <v>2.0887059774144901E-5</v>
+      </c>
+      <c r="C25">
+        <v>2.5052539496126101</v>
+      </c>
+      <c r="D25">
+        <v>1.8829968719792201E-2</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="N25">
+        <v>1071</v>
+      </c>
+      <c r="O25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>23</v>
+      </c>
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="N26">
+        <v>1892</v>
+      </c>
+      <c r="O26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>24</v>
+      </c>
+      <c r="B27">
+        <v>2.1591196456141501E-4</v>
+      </c>
+      <c r="C27">
+        <v>1.7189995203791599</v>
+      </c>
+      <c r="D27">
+        <v>1.20209817420813</v>
+      </c>
+      <c r="E27">
+        <v>0.9</v>
+      </c>
+      <c r="N27">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>25</v>
+      </c>
+      <c r="B28">
+        <v>3.0880065502844102E-4</v>
+      </c>
+      <c r="C28">
+        <v>1.7074022707650001</v>
+      </c>
+      <c r="D28">
+        <v>3.7186641941726502E-4</v>
+      </c>
+      <c r="E28">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>26</v>
+      </c>
+      <c r="E29">
+        <v>0.7</v>
+      </c>
+      <c r="N29">
+        <v>502</v>
+      </c>
+      <c r="O29" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>27</v>
+      </c>
+      <c r="B30">
+        <v>4.60311808037377E-4</v>
+      </c>
+      <c r="C30">
+        <v>1.66187478217667</v>
+      </c>
+      <c r="D30">
+        <v>1.3738648256894E-4</v>
+      </c>
+      <c r="N30">
+        <v>502</v>
+      </c>
+      <c r="O30" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>28</v>
+      </c>
+      <c r="B31">
+        <v>5.86247778425387E-4</v>
+      </c>
+      <c r="C31">
+        <v>1.6630696101604501</v>
+      </c>
+      <c r="D31" s="2">
+        <v>9.39537377217747E-5</v>
+      </c>
+      <c r="M31">
+        <v>0.6</v>
+      </c>
+      <c r="N31">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>29</v>
+      </c>
+      <c r="N32">
+        <v>522</v>
+      </c>
+      <c r="O32" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>30</v>
+      </c>
+      <c r="B33">
+        <v>2.8727643386340098E-4</v>
+      </c>
+      <c r="C33">
+        <v>1.5904189645704501</v>
+      </c>
+      <c r="D33">
+        <v>1.0263197679569199E-4</v>
+      </c>
+      <c r="M33">
+        <v>0</v>
+      </c>
+      <c r="N33">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B34">
+        <v>3.0928717643758302E-4</v>
+      </c>
+      <c r="C34">
+        <v>1.5965904733758101</v>
+      </c>
+      <c r="D34">
+        <v>2.4080124471630401E-4</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="N34">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B35">
+        <v>2.4681495887314401E-4</v>
+      </c>
+      <c r="C35">
+        <v>1.6624759537039799</v>
+      </c>
+      <c r="D35">
+        <v>1.7341179006468701E-4</v>
+      </c>
+      <c r="K35" t="s">
+        <v>77</v>
+      </c>
+      <c r="N35">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E36">
+        <v>0.64</v>
+      </c>
+      <c r="K36" t="s">
+        <v>28</v>
+      </c>
+      <c r="N36">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E37">
+        <v>0.75</v>
+      </c>
+      <c r="N37">
+        <v>550</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5B19FA9-A01B-4042-9995-5A31C36523E9}">
+  <dimension ref="A2:G25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="9.109375" style="4"/>
+    <col min="3" max="3" width="31.88671875" style="4" customWidth="1"/>
+    <col min="4" max="6" width="33.33203125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="4" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
+        <v>11</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>12</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
+        <v>13</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
+        <v>14</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="4">
+        <v>15</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="4">
+        <v>16</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="4">
+        <v>17</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="4">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>